<commit_message>
16 aug rescrape done
</commit_message>
<xml_diff>
--- a/NJSBCL/data/division1_schedule.xlsx
+++ b/NJSBCL/data/division1_schedule.xlsx
@@ -323,7 +323,7 @@
       </c>
       <c t="inlineStr" r="E3">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F3">
@@ -333,22 +333,17 @@
       </c>
       <c t="inlineStr" r="G3">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="H3">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I3">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J3">
-        <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
     </row>
@@ -368,7 +363,7 @@
       </c>
       <c t="inlineStr" r="E4">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F4">
@@ -378,22 +373,22 @@
       </c>
       <c t="inlineStr" r="G4">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="H4">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I4">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">11Spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="J4">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>
@@ -413,7 +408,7 @@
       </c>
       <c t="inlineStr" r="E5">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F5">
@@ -423,22 +418,22 @@
       </c>
       <c t="inlineStr" r="G5">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
       <c t="inlineStr" r="H5">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I5">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="J5">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -458,7 +453,7 @@
       </c>
       <c t="inlineStr" r="E6">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F6">
@@ -468,22 +463,17 @@
       </c>
       <c t="inlineStr" r="G6">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H6">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I6">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J6">
-        <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Samp XI</t>
         </is>
       </c>
     </row>
@@ -503,7 +493,7 @@
       </c>
       <c t="inlineStr" r="E7">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F7">
@@ -513,22 +503,22 @@
       </c>
       <c t="inlineStr" r="G7">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="H7">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I7">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J7">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
     </row>
@@ -548,7 +538,7 @@
       </c>
       <c t="inlineStr" r="E8">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F8">
@@ -558,22 +548,17 @@
       </c>
       <c t="inlineStr" r="G8">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="H8">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I8">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J8">
-        <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
     </row>
@@ -593,7 +578,7 @@
       </c>
       <c t="inlineStr" r="E9">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F9">
@@ -603,22 +588,22 @@
       </c>
       <c t="inlineStr" r="G9">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="H9">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I9">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">FDU Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="J9">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -638,7 +623,7 @@
       </c>
       <c t="inlineStr" r="E10">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F10">
@@ -648,22 +633,22 @@
       </c>
       <c t="inlineStr" r="G10">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H10">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I10">
         <is>
-          <t xml:space="preserve">NJ Braves</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="J10">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -683,7 +668,7 @@
       </c>
       <c t="inlineStr" r="E11">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F11">
@@ -693,22 +678,17 @@
       </c>
       <c t="inlineStr" r="G11">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="H11">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I11">
         <is>
-          <t xml:space="preserve">Blasters</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J11">
-        <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
     </row>
@@ -728,7 +708,7 @@
       </c>
       <c t="inlineStr" r="E12">
         <is>
-          <t xml:space="preserve">08/15/2026</t>
+          <t xml:space="preserve">08/16/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F12">
@@ -738,22 +718,17 @@
       </c>
       <c t="inlineStr" r="G12">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="H12">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I12">
         <is>
-          <t xml:space="preserve">Punjab XI</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J12">
-        <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
     </row>
@@ -773,7 +748,7 @@
       </c>
       <c t="inlineStr" r="E13">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F13">
@@ -788,17 +763,17 @@
       </c>
       <c t="inlineStr" r="H13">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I13">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="J13">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
     </row>
@@ -818,7 +793,7 @@
       </c>
       <c t="inlineStr" r="E14">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F14">
@@ -833,17 +808,17 @@
       </c>
       <c t="inlineStr" r="H14">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I14">
         <is>
-          <t xml:space="preserve">11Spartans</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="J14">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
     </row>
@@ -863,7 +838,7 @@
       </c>
       <c t="inlineStr" r="E15">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F15">
@@ -878,17 +853,17 @@
       </c>
       <c t="inlineStr" r="H15">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I15">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">GCC</t>
         </is>
       </c>
       <c t="inlineStr" r="J15">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
     </row>
@@ -908,7 +883,7 @@
       </c>
       <c t="inlineStr" r="E16">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F16">
@@ -923,17 +898,17 @@
       </c>
       <c t="inlineStr" r="H16">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I16">
         <is>
-          <t xml:space="preserve">Samp XI</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="J16">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
     </row>
@@ -953,7 +928,7 @@
       </c>
       <c t="inlineStr" r="E17">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F17">
@@ -968,17 +943,17 @@
       </c>
       <c t="inlineStr" r="H17">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I17">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="J17">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
     </row>
@@ -998,7 +973,7 @@
       </c>
       <c t="inlineStr" r="E18">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F18">
@@ -1013,17 +988,17 @@
       </c>
       <c t="inlineStr" r="H18">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I18">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="J18">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1018,7 @@
       </c>
       <c t="inlineStr" r="E19">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F19">
@@ -1058,17 +1033,17 @@
       </c>
       <c t="inlineStr" r="H19">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I19">
         <is>
-          <t xml:space="preserve">FDU Giants</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="J19">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1063,7 @@
       </c>
       <c t="inlineStr" r="E20">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F20">
@@ -1103,17 +1078,17 @@
       </c>
       <c t="inlineStr" r="H20">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I20">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="J20">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1108,7 @@
       </c>
       <c t="inlineStr" r="E21">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F21">
@@ -1148,17 +1123,17 @@
       </c>
       <c t="inlineStr" r="H21">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I21">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="J21">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1153,7 @@
       </c>
       <c t="inlineStr" r="E22">
         <is>
-          <t xml:space="preserve">08/16/2026</t>
+          <t xml:space="preserve">08/22/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F22">
@@ -1193,17 +1168,17 @@
       </c>
       <c t="inlineStr" r="H22">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I22">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="J22">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1198,7 @@
       </c>
       <c t="inlineStr" r="E23">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F23">
@@ -1233,22 +1208,22 @@
       </c>
       <c t="inlineStr" r="G23">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="H23">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="I23">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="J23">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1243,7 @@
       </c>
       <c t="inlineStr" r="E24">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F24">
@@ -1278,22 +1253,22 @@
       </c>
       <c t="inlineStr" r="G24">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H24">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I24">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J24">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1288,7 @@
       </c>
       <c t="inlineStr" r="E25">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F25">
@@ -1323,22 +1298,22 @@
       </c>
       <c t="inlineStr" r="G25">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="H25">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I25">
         <is>
-          <t xml:space="preserve">GCC</t>
+          <t xml:space="preserve">NJ Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J25">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1333,7 @@
       </c>
       <c t="inlineStr" r="E26">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F26">
@@ -1368,22 +1343,22 @@
       </c>
       <c t="inlineStr" r="G26">
         <is>
+          <t xml:space="preserve">Storm Riders</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H26">
+        <is>
+          <t xml:space="preserve">Aryans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I26">
+        <is>
+          <t xml:space="preserve">Aryans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J26">
+        <is>
           <t xml:space="preserve">Desi Warriors</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="H26">
-        <is>
-          <t xml:space="preserve">Blue Aces CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I26">
-        <is>
-          <t xml:space="preserve">Desi Warriors</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J26">
-        <is>
-          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1378,7 @@
       </c>
       <c t="inlineStr" r="E27">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F27">
@@ -1413,22 +1388,22 @@
       </c>
       <c t="inlineStr" r="G27">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="H27">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="I27">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="J27">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1423,7 @@
       </c>
       <c t="inlineStr" r="E28">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F28">
@@ -1458,22 +1433,22 @@
       </c>
       <c t="inlineStr" r="G28">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="H28">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="I28">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="J28">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1468,7 @@
       </c>
       <c t="inlineStr" r="E29">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F29">
@@ -1503,22 +1478,22 @@
       </c>
       <c t="inlineStr" r="G29">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="H29">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I29">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="J29">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1513,7 @@
       </c>
       <c t="inlineStr" r="E30">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F30">
@@ -1548,22 +1523,22 @@
       </c>
       <c t="inlineStr" r="G30">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="H30">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="I30">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">NJ Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="J30">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1558,7 @@
       </c>
       <c t="inlineStr" r="E31">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F31">
@@ -1593,22 +1568,22 @@
       </c>
       <c t="inlineStr" r="G31">
         <is>
+          <t xml:space="preserve">Blasters</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H31">
+        <is>
+          <t xml:space="preserve">Jersey Boys</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I31">
+        <is>
+          <t xml:space="preserve">Jersey Boys</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J31">
+        <is>
           <t xml:space="preserve">Youth For Sewa</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="H31">
-        <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I31">
-        <is>
-          <t xml:space="preserve">Youth For Sewa</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J31">
-        <is>
-          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1603,7 @@
       </c>
       <c t="inlineStr" r="E32">
         <is>
-          <t xml:space="preserve">08/22/2026</t>
+          <t xml:space="preserve">08/23/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F32">
@@ -1638,22 +1613,22 @@
       </c>
       <c t="inlineStr" r="G32">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H32">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="I32">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="J32">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1648,7 @@
       </c>
       <c t="inlineStr" r="E33">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F33">
@@ -1688,17 +1663,17 @@
       </c>
       <c t="inlineStr" r="H33">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I33">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="J33">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1693,7 @@
       </c>
       <c t="inlineStr" r="E34">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F34">
@@ -1733,17 +1708,17 @@
       </c>
       <c t="inlineStr" r="H34">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I34">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J34">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1738,7 @@
       </c>
       <c t="inlineStr" r="E35">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F35">
@@ -1778,17 +1753,17 @@
       </c>
       <c t="inlineStr" r="H35">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="I35">
         <is>
-          <t xml:space="preserve">NJ Stars CC</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J35">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1783,7 @@
       </c>
       <c t="inlineStr" r="E36">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F36">
@@ -1823,17 +1798,17 @@
       </c>
       <c t="inlineStr" r="H36">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="I36">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="J36">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1828,7 @@
       </c>
       <c t="inlineStr" r="E37">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F37">
@@ -1868,17 +1843,17 @@
       </c>
       <c t="inlineStr" r="H37">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="I37">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J37">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1873,7 @@
       </c>
       <c t="inlineStr" r="E38">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F38">
@@ -1913,17 +1888,17 @@
       </c>
       <c t="inlineStr" r="H38">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I38">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="J38">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1918,7 @@
       </c>
       <c t="inlineStr" r="E39">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F39">
@@ -1958,17 +1933,17 @@
       </c>
       <c t="inlineStr" r="H39">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="I39">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="J39">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1963,7 @@
       </c>
       <c t="inlineStr" r="E40">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F40">
@@ -2003,17 +1978,17 @@
       </c>
       <c t="inlineStr" r="H40">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="I40">
         <is>
-          <t xml:space="preserve">NJ Tigers</t>
+          <t xml:space="preserve">NJ Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="J40">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2008,7 @@
       </c>
       <c t="inlineStr" r="E41">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F41">
@@ -2048,17 +2023,17 @@
       </c>
       <c t="inlineStr" r="H41">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="I41">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="J41">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2053,7 @@
       </c>
       <c t="inlineStr" r="E42">
         <is>
-          <t xml:space="preserve">08/23/2026</t>
+          <t xml:space="preserve">08/29/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F42">
@@ -2093,17 +2068,17 @@
       </c>
       <c t="inlineStr" r="H42">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="I42">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Punjab XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J42">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2098,7 @@
       </c>
       <c t="inlineStr" r="E43">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F43">
@@ -2133,22 +2108,22 @@
       </c>
       <c t="inlineStr" r="G43">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="H43">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I43">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="J43">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2143,7 @@
       </c>
       <c t="inlineStr" r="E44">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F44">
@@ -2178,22 +2153,22 @@
       </c>
       <c t="inlineStr" r="G44">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="H44">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I44">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Samp XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J44">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2188,7 @@
       </c>
       <c t="inlineStr" r="E45">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F45">
@@ -2223,22 +2198,22 @@
       </c>
       <c t="inlineStr" r="G45">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
       <c t="inlineStr" r="H45">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I45">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J45">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2233,7 @@
       </c>
       <c t="inlineStr" r="E46">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F46">
@@ -2268,22 +2243,22 @@
       </c>
       <c t="inlineStr" r="G46">
         <is>
+          <t xml:space="preserve">Desi Warriors</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H46">
+        <is>
+          <t xml:space="preserve">Maha CC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I46">
+        <is>
+          <t xml:space="preserve">Maha CC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J46">
+        <is>
           <t xml:space="preserve">Storm Riders</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="H46">
-        <is>
-          <t xml:space="preserve">WCC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I46">
-        <is>
-          <t xml:space="preserve">Storm Riders</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J46">
-        <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2278,7 @@
       </c>
       <c t="inlineStr" r="E47">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F47">
@@ -2313,22 +2288,22 @@
       </c>
       <c t="inlineStr" r="G47">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="H47">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I47">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">FDU Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="J47">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2323,7 @@
       </c>
       <c t="inlineStr" r="E48">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F48">
@@ -2358,22 +2333,22 @@
       </c>
       <c t="inlineStr" r="G48">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="H48">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I48">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="J48">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2368,7 @@
       </c>
       <c t="inlineStr" r="E49">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F49">
@@ -2403,22 +2378,22 @@
       </c>
       <c t="inlineStr" r="G49">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="H49">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I49">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="J49">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2413,7 @@
       </c>
       <c t="inlineStr" r="E50">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F50">
@@ -2448,22 +2423,22 @@
       </c>
       <c t="inlineStr" r="G50">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H50">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I50">
         <is>
-          <t xml:space="preserve">NJ Braves</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J50">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2458,7 @@
       </c>
       <c t="inlineStr" r="E51">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F51">
@@ -2493,22 +2468,22 @@
       </c>
       <c t="inlineStr" r="G51">
         <is>
+          <t xml:space="preserve">Youth For Sewa</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H51">
+        <is>
+          <t xml:space="preserve">Gryffindors</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I51">
+        <is>
+          <t xml:space="preserve">Gryffindors</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J51">
+        <is>
           <t xml:space="preserve">Blasters</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="H51">
-        <is>
-          <t xml:space="preserve">Veerans</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I51">
-        <is>
-          <t xml:space="preserve">Blasters</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J51">
-        <is>
-          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2503,7 @@
       </c>
       <c t="inlineStr" r="E52">
         <is>
-          <t xml:space="preserve">08/29/2026</t>
+          <t xml:space="preserve">08/30/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F52">
@@ -2538,22 +2513,22 @@
       </c>
       <c t="inlineStr" r="G52">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="H52">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I52">
         <is>
-          <t xml:space="preserve">Punjab XI</t>
+          <t xml:space="preserve">11Spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="J52">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2548,7 @@
       </c>
       <c t="inlineStr" r="E53">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F53">
@@ -2588,17 +2563,17 @@
       </c>
       <c t="inlineStr" r="H53">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I53">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="J53">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
     </row>
@@ -2618,7 +2593,7 @@
       </c>
       <c t="inlineStr" r="E54">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F54">
@@ -2633,17 +2608,17 @@
       </c>
       <c t="inlineStr" r="H54">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I54">
         <is>
-          <t xml:space="preserve">Samp XI</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="J54">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2638,7 @@
       </c>
       <c t="inlineStr" r="E55">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F55">
@@ -2678,17 +2653,17 @@
       </c>
       <c t="inlineStr" r="H55">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I55">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">GCC</t>
         </is>
       </c>
       <c t="inlineStr" r="J55">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2683,7 @@
       </c>
       <c t="inlineStr" r="E56">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F56">
@@ -2723,17 +2698,17 @@
       </c>
       <c t="inlineStr" r="H56">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I56">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="J56">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2728,7 @@
       </c>
       <c t="inlineStr" r="E57">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F57">
@@ -2768,17 +2743,17 @@
       </c>
       <c t="inlineStr" r="H57">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I57">
         <is>
-          <t xml:space="preserve">FDU Giants</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="J57">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2773,7 @@
       </c>
       <c t="inlineStr" r="E58">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F58">
@@ -2813,17 +2788,17 @@
       </c>
       <c t="inlineStr" r="H58">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I58">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="J58">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2818,7 @@
       </c>
       <c t="inlineStr" r="E59">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F59">
@@ -2858,17 +2833,17 @@
       </c>
       <c t="inlineStr" r="H59">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I59">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="J59">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2863,7 @@
       </c>
       <c t="inlineStr" r="E60">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F60">
@@ -2903,17 +2878,17 @@
       </c>
       <c t="inlineStr" r="H60">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I60">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="J60">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2908,7 @@
       </c>
       <c t="inlineStr" r="E61">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F61">
@@ -2948,17 +2923,17 @@
       </c>
       <c t="inlineStr" r="H61">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I61">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="J61">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2953,7 @@
       </c>
       <c t="inlineStr" r="E62">
         <is>
-          <t xml:space="preserve">08/30/2026</t>
+          <t xml:space="preserve">09/12/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F62">
@@ -2993,17 +2968,17 @@
       </c>
       <c t="inlineStr" r="H62">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I62">
         <is>
-          <t xml:space="preserve">11Spartans</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="J62">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
     </row>
@@ -3023,7 +2998,7 @@
       </c>
       <c t="inlineStr" r="E63">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F63">
@@ -3033,22 +3008,22 @@
       </c>
       <c t="inlineStr" r="G63">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="H63">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I63">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">NJ Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J63">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3043,7 @@
       </c>
       <c t="inlineStr" r="E64">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F64">
@@ -3078,22 +3053,22 @@
       </c>
       <c t="inlineStr" r="G64">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H64">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="I64">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="J64">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3088,7 @@
       </c>
       <c t="inlineStr" r="E65">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F65">
@@ -3123,22 +3098,22 @@
       </c>
       <c t="inlineStr" r="G65">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="H65">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="I65">
         <is>
-          <t xml:space="preserve">GCC</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="J65">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3133,7 @@
       </c>
       <c t="inlineStr" r="E66">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F66">
@@ -3168,22 +3143,22 @@
       </c>
       <c t="inlineStr" r="G66">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="H66">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="I66">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="J66">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3178,7 @@
       </c>
       <c t="inlineStr" r="E67">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F67">
@@ -3213,22 +3188,22 @@
       </c>
       <c t="inlineStr" r="G67">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="H67">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I67">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="J67">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3223,7 @@
       </c>
       <c t="inlineStr" r="E68">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F68">
@@ -3258,22 +3233,22 @@
       </c>
       <c t="inlineStr" r="G68">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="H68">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="I68">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">NJ Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="J68">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3268,7 @@
       </c>
       <c t="inlineStr" r="E69">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F69">
@@ -3303,22 +3278,22 @@
       </c>
       <c t="inlineStr" r="G69">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="H69">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="I69">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="J69">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3313,7 @@
       </c>
       <c t="inlineStr" r="E70">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F70">
@@ -3348,22 +3323,22 @@
       </c>
       <c t="inlineStr" r="G70">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="H70">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="I70">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="J70">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3358,7 @@
       </c>
       <c t="inlineStr" r="E71">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F71">
@@ -3393,22 +3368,22 @@
       </c>
       <c t="inlineStr" r="G71">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="H71">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="I71">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="J71">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3403,7 @@
       </c>
       <c t="inlineStr" r="E72">
         <is>
-          <t xml:space="preserve">09/12/2026</t>
+          <t xml:space="preserve">09/13/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F72">
@@ -3438,22 +3413,22 @@
       </c>
       <c t="inlineStr" r="G72">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H72">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I72">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J72">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3448,7 @@
       </c>
       <c t="inlineStr" r="E73">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F73">
@@ -3488,17 +3463,17 @@
       </c>
       <c t="inlineStr" r="H73">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">Aryans</t>
         </is>
       </c>
       <c t="inlineStr" r="I73">
         <is>
-          <t xml:space="preserve">NJ Stars CC</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="J73">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3493,7 @@
       </c>
       <c t="inlineStr" r="E74">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F74">
@@ -3533,17 +3508,17 @@
       </c>
       <c t="inlineStr" r="H74">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">WCC</t>
         </is>
       </c>
       <c t="inlineStr" r="I74">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J74">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3538,7 @@
       </c>
       <c t="inlineStr" r="E75">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F75">
@@ -3578,17 +3553,17 @@
       </c>
       <c t="inlineStr" r="H75">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Plainsboro Eagles</t>
         </is>
       </c>
       <c t="inlineStr" r="I75">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J75">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3583,7 @@
       </c>
       <c t="inlineStr" r="E76">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F76">
@@ -3623,17 +3598,17 @@
       </c>
       <c t="inlineStr" r="H76">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I76">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="J76">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3628,7 @@
       </c>
       <c t="inlineStr" r="E77">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F77">
@@ -3668,17 +3643,17 @@
       </c>
       <c t="inlineStr" r="H77">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Nj Tigers</t>
         </is>
       </c>
       <c t="inlineStr" r="I77">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J77">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3673,7 @@
       </c>
       <c t="inlineStr" r="E78">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F78">
@@ -3713,17 +3688,17 @@
       </c>
       <c t="inlineStr" r="H78">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">Jersey Boys</t>
         </is>
       </c>
       <c t="inlineStr" r="I78">
         <is>
-          <t xml:space="preserve">NJ Tigers</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="J78">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3718,7 @@
       </c>
       <c t="inlineStr" r="E79">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F79">
@@ -3758,17 +3733,17 @@
       </c>
       <c t="inlineStr" r="H79">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Veerans</t>
         </is>
       </c>
       <c t="inlineStr" r="I79">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="J79">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3763,7 @@
       </c>
       <c t="inlineStr" r="E80">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F80">
@@ -3803,17 +3778,17 @@
       </c>
       <c t="inlineStr" r="H80">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Edison Rebelz</t>
         </is>
       </c>
       <c t="inlineStr" r="I80">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">NJ Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="J80">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3808,7 @@
       </c>
       <c t="inlineStr" r="E81">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F81">
@@ -3848,17 +3823,17 @@
       </c>
       <c t="inlineStr" r="H81">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I81">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="J81">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3853,7 @@
       </c>
       <c t="inlineStr" r="E82">
         <is>
-          <t xml:space="preserve">09/13/2026</t>
+          <t xml:space="preserve">09/19/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F82">
@@ -3893,17 +3868,17 @@
       </c>
       <c t="inlineStr" r="H82">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I82">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Punjab XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J82">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3898,7 @@
       </c>
       <c t="inlineStr" r="E83">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F83">
@@ -3933,22 +3908,22 @@
       </c>
       <c t="inlineStr" r="G83">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Team Highlanders</t>
         </is>
       </c>
       <c t="inlineStr" r="H83">
         <is>
-          <t xml:space="preserve">Aryans</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I83">
         <is>
-          <t xml:space="preserve">Pway Lions</t>
+          <t xml:space="preserve">Blue Aces CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J83">
         <is>
-          <t xml:space="preserve">11spartans</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3943,7 @@
       </c>
       <c t="inlineStr" r="E84">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F84">
@@ -3978,22 +3953,22 @@
       </c>
       <c t="inlineStr" r="G84">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Samudhra Gladiators</t>
         </is>
       </c>
       <c t="inlineStr" r="H84">
         <is>
-          <t xml:space="preserve">WCC</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I84">
         <is>
-          <t xml:space="preserve">Gujarat United XI</t>
+          <t xml:space="preserve">Maha CC</t>
         </is>
       </c>
       <c t="inlineStr" r="J84">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
     </row>
@@ -4013,7 +3988,7 @@
       </c>
       <c t="inlineStr" r="E85">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F85">
@@ -4023,22 +3998,22 @@
       </c>
       <c t="inlineStr" r="G85">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">Gcc</t>
         </is>
       </c>
       <c t="inlineStr" r="H85">
         <is>
-          <t xml:space="preserve">Plainsboro Eagles</t>
+          <t xml:space="preserve">Fdu Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="I85">
         <is>
-          <t xml:space="preserve">Newport CC</t>
+          <t xml:space="preserve">FDU Giants</t>
         </is>
       </c>
       <c t="inlineStr" r="J85">
         <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4033,7 @@
       </c>
       <c t="inlineStr" r="E86">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F86">
@@ -4068,22 +4043,22 @@
       </c>
       <c t="inlineStr" r="G86">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Desi Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H86">
         <is>
-          <t xml:space="preserve">Jetha 11</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="I86">
         <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">Juggernaut</t>
         </is>
       </c>
       <c t="inlineStr" r="J86">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4078,7 @@
       </c>
       <c t="inlineStr" r="E87">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F87">
@@ -4113,22 +4088,22 @@
       </c>
       <c t="inlineStr" r="G87">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">Sreeshti</t>
         </is>
       </c>
       <c t="inlineStr" r="H87">
         <is>
-          <t xml:space="preserve">Nj Tigers</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="I87">
         <is>
-          <t xml:space="preserve">Mercer Challengers</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c t="inlineStr" r="J87">
         <is>
-          <t xml:space="preserve">Juggernaut</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4123,7 @@
       </c>
       <c t="inlineStr" r="E88">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F88">
@@ -4158,22 +4133,22 @@
       </c>
       <c t="inlineStr" r="G88">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Hudson Hurricanes</t>
         </is>
       </c>
       <c t="inlineStr" r="H88">
         <is>
-          <t xml:space="preserve">Jersey Boys</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="I88">
         <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
+          <t xml:space="preserve">Piscataway Avengers</t>
         </is>
       </c>
       <c t="inlineStr" r="J88">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4168,7 @@
       </c>
       <c t="inlineStr" r="E89">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F89">
@@ -4203,22 +4178,22 @@
       </c>
       <c t="inlineStr" r="G89">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Falcons</t>
         </is>
       </c>
       <c t="inlineStr" r="H89">
         <is>
-          <t xml:space="preserve">Veerans</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="I89">
         <is>
-          <t xml:space="preserve">Jersey Titans</t>
+          <t xml:space="preserve">Gryffindors</t>
         </is>
       </c>
       <c t="inlineStr" r="J89">
         <is>
-          <t xml:space="preserve">Maha CC</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4213,7 @@
       </c>
       <c t="inlineStr" r="E90">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F90">
@@ -4248,22 +4223,22 @@
       </c>
       <c t="inlineStr" r="G90">
         <is>
-          <t xml:space="preserve">Nj Braves</t>
+          <t xml:space="preserve">Warriors</t>
         </is>
       </c>
       <c t="inlineStr" r="H90">
         <is>
-          <t xml:space="preserve">Edison Rebelz</t>
+          <t xml:space="preserve">11spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="I90">
         <is>
-          <t xml:space="preserve">NJ Braves</t>
+          <t xml:space="preserve">11Spartans</t>
         </is>
       </c>
       <c t="inlineStr" r="J90">
         <is>
-          <t xml:space="preserve">Blue Aces CC</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4258,7 @@
       </c>
       <c t="inlineStr" r="E91">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F91">
@@ -4293,22 +4268,22 @@
       </c>
       <c t="inlineStr" r="G91">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Youth For Sewa</t>
         </is>
       </c>
       <c t="inlineStr" r="H91">
         <is>
-          <t xml:space="preserve">Parsippany Phoenix XI</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="I91">
         <is>
-          <t xml:space="preserve">Blasters</t>
+          <t xml:space="preserve">Rowdy Rebels</t>
         </is>
       </c>
       <c t="inlineStr" r="J91">
         <is>
-          <t xml:space="preserve">SAMP XI</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4303,7 @@
       </c>
       <c t="inlineStr" r="E92">
         <is>
-          <t xml:space="preserve">09/19/2026</t>
+          <t xml:space="preserve">09/20/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F92">
@@ -4338,22 +4313,22 @@
       </c>
       <c t="inlineStr" r="G92">
         <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">RHG</t>
         </is>
       </c>
       <c t="inlineStr" r="H92">
         <is>
-          <t xml:space="preserve">Nj Stars CC</t>
+          <t xml:space="preserve">SAMP XI</t>
         </is>
       </c>
       <c t="inlineStr" r="I92">
         <is>
-          <t xml:space="preserve">Punjab XI</t>
+          <t xml:space="preserve">Samp XI</t>
         </is>
       </c>
       <c t="inlineStr" r="J92">
         <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4348,7 @@
       </c>
       <c t="inlineStr" r="E93">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F93">
@@ -4383,22 +4358,22 @@
       </c>
       <c t="inlineStr" r="G93">
         <is>
-          <t xml:space="preserve">Team Highlanders</t>
+          <t xml:space="preserve">PUNJAB XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H93">
         <is>
+          <t xml:space="preserve">Jersey Boys</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I93">
+        <is>
+          <t xml:space="preserve">Punjab XI</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J93">
+        <is>
           <t xml:space="preserve">Blue Aces CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I93">
-        <is>
-          <t xml:space="preserve">Blue Aces CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J93">
-        <is>
-          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
     </row>
@@ -4418,7 +4393,7 @@
       </c>
       <c t="inlineStr" r="E94">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F94">
@@ -4428,22 +4403,22 @@
       </c>
       <c t="inlineStr" r="G94">
         <is>
-          <t xml:space="preserve">Samudhra Gladiators</t>
+          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
       <c t="inlineStr" r="H94">
         <is>
+          <t xml:space="preserve">Nj Tigers</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I94">
+        <is>
+          <t xml:space="preserve">Blasters</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J94">
+        <is>
           <t xml:space="preserve">Maha CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I94">
-        <is>
-          <t xml:space="preserve">Maha CC</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J94">
-        <is>
-          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4438,7 @@
       </c>
       <c t="inlineStr" r="E95">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F95">
@@ -4473,22 +4448,17 @@
       </c>
       <c t="inlineStr" r="G95">
         <is>
-          <t xml:space="preserve">Gcc</t>
+          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
       <c t="inlineStr" r="H95">
         <is>
-          <t xml:space="preserve">Fdu Giants</t>
+          <t xml:space="preserve">Jetha 11</t>
         </is>
       </c>
       <c t="inlineStr" r="I95">
         <is>
-          <t xml:space="preserve">FDU Giants</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J95">
-        <is>
-          <t xml:space="preserve">Storm Riders</t>
+          <t xml:space="preserve">NJ Braves</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4478,7 @@
       </c>
       <c t="inlineStr" r="E96">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F96">
@@ -4518,22 +4488,22 @@
       </c>
       <c t="inlineStr" r="G96">
         <is>
-          <t xml:space="preserve">Desi Warriors</t>
+          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
       <c t="inlineStr" r="H96">
         <is>
+          <t xml:space="preserve">Plainsboro Eagles</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I96">
+        <is>
+          <t xml:space="preserve">Jersey Titans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J96">
+        <is>
           <t xml:space="preserve">Juggernaut</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I96">
-        <is>
-          <t xml:space="preserve">Juggernaut</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J96">
-        <is>
-          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4523,7 @@
       </c>
       <c t="inlineStr" r="E97">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F97">
@@ -4563,22 +4533,22 @@
       </c>
       <c t="inlineStr" r="G97">
         <is>
-          <t xml:space="preserve">Sreeshti</t>
+          <t xml:space="preserve">Plainsboro Knights</t>
         </is>
       </c>
       <c t="inlineStr" r="H97">
         <is>
+          <t xml:space="preserve">WCC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I97">
+        <is>
+          <t xml:space="preserve">Plainsboro Knights</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J97">
+        <is>
           <t xml:space="preserve">F5</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I97">
-        <is>
-          <t xml:space="preserve">F5</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J97">
-        <is>
-          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4568,7 @@
       </c>
       <c t="inlineStr" r="E98">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F98">
@@ -4608,22 +4578,22 @@
       </c>
       <c t="inlineStr" r="G98">
         <is>
-          <t xml:space="preserve">Hudson Hurricanes</t>
+          <t xml:space="preserve">Mercer Challengers</t>
         </is>
       </c>
       <c t="inlineStr" r="H98">
         <is>
+          <t xml:space="preserve">Aryans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I98">
+        <is>
+          <t xml:space="preserve">Mercer Challengers</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J98">
+        <is>
           <t xml:space="preserve">Piscataway Avengers</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I98">
-        <is>
-          <t xml:space="preserve">Piscataway Avengers</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J98">
-        <is>
-          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4613,7 @@
       </c>
       <c t="inlineStr" r="E99">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F99">
@@ -4653,22 +4623,17 @@
       </c>
       <c t="inlineStr" r="G99">
         <is>
-          <t xml:space="preserve">Falcons</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
       <c t="inlineStr" r="H99">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
+          <t xml:space="preserve">Nj Stars CC</t>
         </is>
       </c>
       <c t="inlineStr" r="I99">
         <is>
-          <t xml:space="preserve">Gryffindors</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J99">
-        <is>
-          <t xml:space="preserve">PUNJAB XI</t>
+          <t xml:space="preserve">Storm Riders</t>
         </is>
       </c>
     </row>
@@ -4688,7 +4653,7 @@
       </c>
       <c t="inlineStr" r="E100">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F100">
@@ -4698,22 +4663,22 @@
       </c>
       <c t="inlineStr" r="G100">
         <is>
-          <t xml:space="preserve">Warriors</t>
+          <t xml:space="preserve">Newport CC</t>
         </is>
       </c>
       <c t="inlineStr" r="H100">
         <is>
+          <t xml:space="preserve">Parsippany Phoenix XI</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I100">
+        <is>
+          <t xml:space="preserve">Newport CC</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J100">
+        <is>
           <t xml:space="preserve">11spartans</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I100">
-        <is>
-          <t xml:space="preserve">11Spartans</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J100">
-        <is>
-          <t xml:space="preserve">Blasters</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4698,7 @@
       </c>
       <c t="inlineStr" r="E101">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F101">
@@ -4743,22 +4708,22 @@
       </c>
       <c t="inlineStr" r="G101">
         <is>
-          <t xml:space="preserve">Youth For Sewa</t>
+          <t xml:space="preserve">Gujarat United XI</t>
         </is>
       </c>
       <c t="inlineStr" r="H101">
         <is>
+          <t xml:space="preserve">Edison Rebelz</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I101">
+        <is>
+          <t xml:space="preserve">Gujarat United XI</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J101">
+        <is>
           <t xml:space="preserve">Rowdy Rebels</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I101">
-        <is>
-          <t xml:space="preserve">Rowdy Rebels</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J101">
-        <is>
-          <t xml:space="preserve">Nj Braves</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4743,7 @@
       </c>
       <c t="inlineStr" r="E102">
         <is>
-          <t xml:space="preserve">09/20/2026</t>
+          <t xml:space="preserve">08/15/2026</t>
         </is>
       </c>
       <c t="inlineStr" r="F102">
@@ -4788,22 +4753,22 @@
       </c>
       <c t="inlineStr" r="G102">
         <is>
-          <t xml:space="preserve">RHG</t>
+          <t xml:space="preserve">Pway Lions</t>
         </is>
       </c>
       <c t="inlineStr" r="H102">
         <is>
+          <t xml:space="preserve">Veerans</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="I102">
+        <is>
+          <t xml:space="preserve">Pway Lions</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="J102">
+        <is>
           <t xml:space="preserve">SAMP XI</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="I102">
-        <is>
-          <t xml:space="preserve">Samp XI</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="J102">
-        <is>
-          <t xml:space="preserve">Jersey Titans</t>
         </is>
       </c>
     </row>

</xml_diff>